<commit_message>
--- Auto Git Commit ---
</commit_message>
<xml_diff>
--- a/정렬결과.xlsx
+++ b/정렬결과.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
   <si>
     <t>경로</t>
   </si>
@@ -29,6 +29,9 @@
   </si>
   <si>
     <t>시간4</t>
+  </si>
+  <si>
+    <t>라벨</t>
   </si>
   <si>
     <t>시간합</t>
@@ -599,10 +602,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -621,10 +624,13 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2">
         <v>23</v>
@@ -639,12 +645,15 @@
         <v>1</v>
       </c>
       <c r="F2">
+        <v>13</v>
+      </c>
+      <c r="G2">
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3">
         <v>20</v>
@@ -659,12 +668,15 @@
         <v>5</v>
       </c>
       <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3">
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4">
         <v>23</v>
@@ -679,12 +691,15 @@
         <v>4</v>
       </c>
       <c r="F4">
+        <v>3</v>
+      </c>
+      <c r="G4">
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B5">
         <v>23</v>
@@ -699,12 +714,15 @@
         <v>4</v>
       </c>
       <c r="F5">
+        <v>4</v>
+      </c>
+      <c r="G5">
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B6">
         <v>23</v>
@@ -719,12 +737,15 @@
         <v>4</v>
       </c>
       <c r="F6">
+        <v>6</v>
+      </c>
+      <c r="G6">
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B7">
         <v>23</v>
@@ -739,12 +760,15 @@
         <v>1</v>
       </c>
       <c r="F7">
+        <v>28</v>
+      </c>
+      <c r="G7">
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8">
         <v>23</v>
@@ -759,12 +783,15 @@
         <v>2</v>
       </c>
       <c r="F8">
+        <v>16</v>
+      </c>
+      <c r="G8">
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B9">
         <v>23</v>
@@ -779,12 +806,15 @@
         <v>5</v>
       </c>
       <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B10">
         <v>20</v>
@@ -799,12 +829,15 @@
         <v>1</v>
       </c>
       <c r="F10">
+        <v>12</v>
+      </c>
+      <c r="G10">
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B11">
         <v>23</v>
@@ -819,12 +852,15 @@
         <v>2</v>
       </c>
       <c r="F11">
+        <v>26</v>
+      </c>
+      <c r="G11">
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B12">
         <v>20</v>
@@ -839,12 +875,15 @@
         <v>5</v>
       </c>
       <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B13">
         <v>20</v>
@@ -859,12 +898,15 @@
         <v>2</v>
       </c>
       <c r="F13">
+        <v>10</v>
+      </c>
+      <c r="G13">
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B14">
         <v>23</v>
@@ -879,12 +921,15 @@
         <v>1</v>
       </c>
       <c r="F14">
+        <v>23</v>
+      </c>
+      <c r="G14">
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B15">
         <v>23</v>
@@ -899,12 +944,15 @@
         <v>5</v>
       </c>
       <c r="F15">
+        <v>13</v>
+      </c>
+      <c r="G15">
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B16">
         <v>23</v>
@@ -919,12 +967,15 @@
         <v>2</v>
       </c>
       <c r="F16">
+        <v>26</v>
+      </c>
+      <c r="G16">
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:7">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B17">
         <v>23</v>
@@ -939,12 +990,15 @@
         <v>5</v>
       </c>
       <c r="F17">
+        <v>32</v>
+      </c>
+      <c r="G17">
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:7">
       <c r="A18" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B18">
         <v>23</v>
@@ -959,12 +1013,15 @@
         <v>5</v>
       </c>
       <c r="F18">
+        <v>16</v>
+      </c>
+      <c r="G18">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:7">
       <c r="A19" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B19">
         <v>23</v>
@@ -979,12 +1036,15 @@
         <v>5</v>
       </c>
       <c r="F19">
+        <v>23</v>
+      </c>
+      <c r="G19">
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:7">
       <c r="A20" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B20">
         <v>21</v>
@@ -999,12 +1059,15 @@
         <v>5</v>
       </c>
       <c r="F20">
+        <v>36</v>
+      </c>
+      <c r="G20">
         <v>35</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:7">
       <c r="A21" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B21">
         <v>23</v>
@@ -1019,12 +1082,15 @@
         <v>5</v>
       </c>
       <c r="F21">
+        <v>7</v>
+      </c>
+      <c r="G21">
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:7">
       <c r="A22" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B22">
         <v>23</v>
@@ -1039,12 +1105,15 @@
         <v>1</v>
       </c>
       <c r="F22">
+        <v>22</v>
+      </c>
+      <c r="G22">
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:7">
       <c r="A23" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B23">
         <v>23</v>
@@ -1059,12 +1128,15 @@
         <v>1</v>
       </c>
       <c r="F23">
+        <v>29</v>
+      </c>
+      <c r="G23">
         <v>35</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:7">
       <c r="A24" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B24">
         <v>23</v>
@@ -1079,12 +1151,15 @@
         <v>5</v>
       </c>
       <c r="F24">
+        <v>34</v>
+      </c>
+      <c r="G24">
         <v>35</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:7">
       <c r="A25" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B25">
         <v>20</v>
@@ -1099,12 +1174,15 @@
         <v>5</v>
       </c>
       <c r="F25">
+        <v>8</v>
+      </c>
+      <c r="G25">
         <v>36</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:7">
       <c r="A26" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B26">
         <v>23</v>
@@ -1119,12 +1197,15 @@
         <v>6</v>
       </c>
       <c r="F26">
+        <v>8</v>
+      </c>
+      <c r="G26">
         <v>36</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:7">
       <c r="A27" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B27">
         <v>23</v>
@@ -1139,73 +1220,85 @@
         <v>2</v>
       </c>
       <c r="F27">
+        <v>20</v>
+      </c>
+      <c r="G27">
         <v>36</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:7">
       <c r="A28" t="s">
+        <v>33</v>
+      </c>
+      <c r="B28">
+        <v>23</v>
+      </c>
+      <c r="C28">
+        <v>4</v>
+      </c>
+      <c r="D28">
+        <v>4</v>
+      </c>
+      <c r="E28">
+        <v>5</v>
+      </c>
+      <c r="F28">
+        <v>26</v>
+      </c>
+      <c r="G28">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" t="s">
+        <v>34</v>
+      </c>
+      <c r="B29">
+        <v>23</v>
+      </c>
+      <c r="C29">
+        <v>6</v>
+      </c>
+      <c r="D29">
+        <v>5</v>
+      </c>
+      <c r="E29">
+        <v>2</v>
+      </c>
+      <c r="F29">
         <v>32</v>
       </c>
-      <c r="B28">
-        <v>23</v>
-      </c>
-      <c r="C28">
-        <v>4</v>
-      </c>
-      <c r="D28">
-        <v>4</v>
-      </c>
-      <c r="E28">
-        <v>5</v>
-      </c>
-      <c r="F28">
+      <c r="G29">
         <v>36</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
-      <c r="A29" t="s">
-        <v>33</v>
-      </c>
-      <c r="B29">
-        <v>23</v>
-      </c>
-      <c r="C29">
-        <v>6</v>
-      </c>
-      <c r="D29">
-        <v>5</v>
-      </c>
-      <c r="E29">
-        <v>2</v>
-      </c>
-      <c r="F29">
+    <row r="30" spans="1:7">
+      <c r="A30" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30">
+        <v>23</v>
+      </c>
+      <c r="C30">
+        <v>2</v>
+      </c>
+      <c r="D30">
+        <v>5</v>
+      </c>
+      <c r="E30">
+        <v>6</v>
+      </c>
+      <c r="F30">
+        <v>35</v>
+      </c>
+      <c r="G30">
         <v>36</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
-      <c r="A30" t="s">
-        <v>34</v>
-      </c>
-      <c r="B30">
-        <v>23</v>
-      </c>
-      <c r="C30">
-        <v>2</v>
-      </c>
-      <c r="D30">
-        <v>5</v>
-      </c>
-      <c r="E30">
-        <v>6</v>
-      </c>
-      <c r="F30">
+    <row r="31" spans="1:7">
+      <c r="A31" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="31" spans="1:6">
-      <c r="A31" t="s">
-        <v>35</v>
-      </c>
       <c r="B31">
         <v>23</v>
       </c>
@@ -1219,12 +1312,15 @@
         <v>11</v>
       </c>
       <c r="F31">
+        <v>2</v>
+      </c>
+      <c r="G31">
         <v>37</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:7">
       <c r="A32" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B32">
         <v>23</v>
@@ -1239,12 +1335,15 @@
         <v>7</v>
       </c>
       <c r="F32">
+        <v>10</v>
+      </c>
+      <c r="G32">
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:7">
       <c r="A33" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B33">
         <v>23</v>
@@ -1259,52 +1358,61 @@
         <v>7</v>
       </c>
       <c r="F33">
+        <v>29</v>
+      </c>
+      <c r="G33">
         <v>37</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:7">
       <c r="A34" t="s">
+        <v>39</v>
+      </c>
+      <c r="B34">
+        <v>23</v>
+      </c>
+      <c r="C34">
+        <v>4</v>
+      </c>
+      <c r="D34">
+        <v>5</v>
+      </c>
+      <c r="E34">
+        <v>5</v>
+      </c>
+      <c r="F34">
+        <v>17</v>
+      </c>
+      <c r="G34">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35" t="s">
+        <v>40</v>
+      </c>
+      <c r="B35">
+        <v>23</v>
+      </c>
+      <c r="C35">
+        <v>4</v>
+      </c>
+      <c r="D35">
+        <v>5</v>
+      </c>
+      <c r="E35">
+        <v>6</v>
+      </c>
+      <c r="F35">
+        <v>18</v>
+      </c>
+      <c r="G35">
         <v>38</v>
       </c>
-      <c r="B34">
-        <v>23</v>
-      </c>
-      <c r="C34">
-        <v>4</v>
-      </c>
-      <c r="D34">
-        <v>5</v>
-      </c>
-      <c r="E34">
-        <v>5</v>
-      </c>
-      <c r="F34">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6">
-      <c r="A35" t="s">
-        <v>39</v>
-      </c>
-      <c r="B35">
-        <v>23</v>
-      </c>
-      <c r="C35">
-        <v>4</v>
-      </c>
-      <c r="D35">
-        <v>5</v>
-      </c>
-      <c r="E35">
-        <v>6</v>
-      </c>
-      <c r="F35">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6">
+    </row>
+    <row r="36" spans="1:7">
       <c r="A36" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B36">
         <v>23</v>
@@ -1319,12 +1427,15 @@
         <v>1</v>
       </c>
       <c r="F36">
+        <v>32</v>
+      </c>
+      <c r="G36">
         <v>39</v>
       </c>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:7">
       <c r="A37" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B37">
         <v>23</v>
@@ -1339,12 +1450,15 @@
         <v>7</v>
       </c>
       <c r="F37">
+        <v>20</v>
+      </c>
+      <c r="G37">
         <v>39</v>
       </c>
     </row>
-    <row r="38" spans="1:6">
+    <row r="38" spans="1:7">
       <c r="A38" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B38">
         <v>23</v>
@@ -1359,12 +1473,15 @@
         <v>5</v>
       </c>
       <c r="F38">
+        <v>32</v>
+      </c>
+      <c r="G38">
         <v>40</v>
       </c>
     </row>
-    <row r="39" spans="1:6">
+    <row r="39" spans="1:7">
       <c r="A39" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B39">
         <v>20</v>
@@ -1379,12 +1496,15 @@
         <v>1</v>
       </c>
       <c r="F39">
+        <v>5</v>
+      </c>
+      <c r="G39">
         <v>40</v>
       </c>
     </row>
-    <row r="40" spans="1:6">
+    <row r="40" spans="1:7">
       <c r="A40" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B40">
         <v>20</v>
@@ -1399,12 +1519,15 @@
         <v>1</v>
       </c>
       <c r="F40">
+        <v>9</v>
+      </c>
+      <c r="G40">
         <v>40</v>
       </c>
     </row>
-    <row r="41" spans="1:6">
+    <row r="41" spans="1:7">
       <c r="A41" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B41">
         <v>23</v>
@@ -1419,12 +1542,15 @@
         <v>2</v>
       </c>
       <c r="F41">
+        <v>36</v>
+      </c>
+      <c r="G41">
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:6">
+    <row r="42" spans="1:7">
       <c r="A42" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B42">
         <v>23</v>
@@ -1439,12 +1565,15 @@
         <v>5</v>
       </c>
       <c r="F42">
+        <v>18</v>
+      </c>
+      <c r="G42">
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="1:6">
+    <row r="43" spans="1:7">
       <c r="A43" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B43">
         <v>20</v>
@@ -1459,12 +1588,15 @@
         <v>2</v>
       </c>
       <c r="F43">
+        <v>3</v>
+      </c>
+      <c r="G43">
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="1:6">
+    <row r="44" spans="1:7">
       <c r="A44" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B44">
         <v>23</v>
@@ -1479,12 +1611,15 @@
         <v>11</v>
       </c>
       <c r="F44">
+        <v>33</v>
+      </c>
+      <c r="G44">
         <v>41</v>
       </c>
     </row>
-    <row r="45" spans="1:6">
+    <row r="45" spans="1:7">
       <c r="A45" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B45">
         <v>20</v>
@@ -1499,12 +1634,15 @@
         <v>2</v>
       </c>
       <c r="F45">
+        <v>7</v>
+      </c>
+      <c r="G45">
         <v>41</v>
       </c>
     </row>
-    <row r="46" spans="1:6">
+    <row r="46" spans="1:7">
       <c r="A46" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B46">
         <v>23</v>
@@ -1519,12 +1657,15 @@
         <v>11</v>
       </c>
       <c r="F46">
+        <v>6</v>
+      </c>
+      <c r="G46">
         <v>41</v>
       </c>
     </row>
-    <row r="47" spans="1:6">
+    <row r="47" spans="1:7">
       <c r="A47" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B47">
         <v>23</v>
@@ -1539,12 +1680,15 @@
         <v>7</v>
       </c>
       <c r="F47">
+        <v>13</v>
+      </c>
+      <c r="G47">
         <v>41</v>
       </c>
     </row>
-    <row r="48" spans="1:6">
+    <row r="48" spans="1:7">
       <c r="A48" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B48">
         <v>23</v>
@@ -1559,12 +1703,15 @@
         <v>1</v>
       </c>
       <c r="F48">
+        <v>19</v>
+      </c>
+      <c r="G48">
         <v>42</v>
       </c>
     </row>
-    <row r="49" spans="1:6">
+    <row r="49" spans="1:7">
       <c r="A49" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B49">
         <v>23</v>
@@ -1579,12 +1726,15 @@
         <v>8</v>
       </c>
       <c r="F49">
+        <v>10</v>
+      </c>
+      <c r="G49">
         <v>42</v>
       </c>
     </row>
-    <row r="50" spans="1:6">
+    <row r="50" spans="1:7">
       <c r="A50" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B50">
         <v>23</v>
@@ -1599,12 +1749,15 @@
         <v>8</v>
       </c>
       <c r="F50">
+        <v>11</v>
+      </c>
+      <c r="G50">
         <v>42</v>
       </c>
     </row>
-    <row r="51" spans="1:6">
+    <row r="51" spans="1:7">
       <c r="A51" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B51">
         <v>23</v>
@@ -1619,12 +1772,15 @@
         <v>5</v>
       </c>
       <c r="F51">
+        <v>36</v>
+      </c>
+      <c r="G51">
         <v>43</v>
       </c>
     </row>
-    <row r="52" spans="1:6">
+    <row r="52" spans="1:7">
       <c r="A52" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B52">
         <v>23</v>
@@ -1639,12 +1795,15 @@
         <v>2</v>
       </c>
       <c r="F52">
+        <v>17</v>
+      </c>
+      <c r="G52">
         <v>43</v>
       </c>
     </row>
-    <row r="53" spans="1:6">
+    <row r="53" spans="1:7">
       <c r="A53" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B53">
         <v>20</v>
@@ -1659,12 +1818,15 @@
         <v>7</v>
       </c>
       <c r="F53">
+        <v>11</v>
+      </c>
+      <c r="G53">
         <v>43</v>
       </c>
     </row>
-    <row r="54" spans="1:6">
+    <row r="54" spans="1:7">
       <c r="A54" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B54">
         <v>23</v>
@@ -1679,12 +1841,15 @@
         <v>7</v>
       </c>
       <c r="F54">
+        <v>27</v>
+      </c>
+      <c r="G54">
         <v>43</v>
       </c>
     </row>
-    <row r="55" spans="1:6">
+    <row r="55" spans="1:7">
       <c r="A55" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B55">
         <v>23</v>
@@ -1699,12 +1864,15 @@
         <v>11</v>
       </c>
       <c r="F55">
+        <v>16</v>
+      </c>
+      <c r="G55">
         <v>43</v>
       </c>
     </row>
-    <row r="56" spans="1:6">
+    <row r="56" spans="1:7">
       <c r="A56" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B56">
         <v>20</v>
@@ -1719,12 +1887,15 @@
         <v>5</v>
       </c>
       <c r="F56">
+        <v>2</v>
+      </c>
+      <c r="G56">
         <v>44</v>
       </c>
     </row>
-    <row r="57" spans="1:6">
+    <row r="57" spans="1:7">
       <c r="A57" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B57">
         <v>23</v>
@@ -1739,12 +1910,15 @@
         <v>8</v>
       </c>
       <c r="F57">
+        <v>30</v>
+      </c>
+      <c r="G57">
         <v>44</v>
       </c>
     </row>
-    <row r="58" spans="1:6">
+    <row r="58" spans="1:7">
       <c r="A58" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B58">
         <v>20</v>
@@ -1759,12 +1933,15 @@
         <v>5</v>
       </c>
       <c r="F58">
+        <v>6</v>
+      </c>
+      <c r="G58">
         <v>44</v>
       </c>
     </row>
-    <row r="59" spans="1:6">
+    <row r="59" spans="1:7">
       <c r="A59" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B59">
         <v>20</v>
@@ -1779,12 +1956,15 @@
         <v>8</v>
       </c>
       <c r="F59">
+        <v>14</v>
+      </c>
+      <c r="G59">
         <v>44</v>
       </c>
     </row>
-    <row r="60" spans="1:6">
+    <row r="60" spans="1:7">
       <c r="A60" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B60">
         <v>20</v>
@@ -1799,12 +1979,15 @@
         <v>8</v>
       </c>
       <c r="F60">
+        <v>15</v>
+      </c>
+      <c r="G60">
         <v>44</v>
       </c>
     </row>
-    <row r="61" spans="1:6">
+    <row r="61" spans="1:7">
       <c r="A61" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B61">
         <v>23</v>
@@ -1819,12 +2002,15 @@
         <v>8</v>
       </c>
       <c r="F61">
+        <v>31</v>
+      </c>
+      <c r="G61">
         <v>44</v>
       </c>
     </row>
-    <row r="62" spans="1:6">
+    <row r="62" spans="1:7">
       <c r="A62" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B62">
         <v>23</v>
@@ -1839,12 +2025,15 @@
         <v>7</v>
       </c>
       <c r="F62">
+        <v>23</v>
+      </c>
+      <c r="G62">
         <v>45</v>
       </c>
     </row>
-    <row r="63" spans="1:6">
+    <row r="63" spans="1:7">
       <c r="A63" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B63">
         <v>23</v>
@@ -1859,12 +2048,15 @@
         <v>8</v>
       </c>
       <c r="F63">
+        <v>20</v>
+      </c>
+      <c r="G63">
         <v>46</v>
       </c>
     </row>
-    <row r="64" spans="1:6">
+    <row r="64" spans="1:7">
       <c r="A64" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B64">
         <v>23</v>
@@ -1879,12 +2071,15 @@
         <v>8</v>
       </c>
       <c r="F64">
+        <v>21</v>
+      </c>
+      <c r="G64">
         <v>46</v>
       </c>
     </row>
-    <row r="65" spans="1:6">
+    <row r="65" spans="1:7">
       <c r="A65" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B65">
         <v>23</v>
@@ -1899,12 +2094,15 @@
         <v>5</v>
       </c>
       <c r="F65">
+        <v>16</v>
+      </c>
+      <c r="G65">
         <v>46</v>
       </c>
     </row>
-    <row r="66" spans="1:6">
+    <row r="66" spans="1:7">
       <c r="A66" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B66">
         <v>23</v>
@@ -1919,12 +2117,15 @@
         <v>7</v>
       </c>
       <c r="F66">
+        <v>21</v>
+      </c>
+      <c r="G66">
         <v>47</v>
       </c>
     </row>
-    <row r="67" spans="1:6">
+    <row r="67" spans="1:7">
       <c r="A67" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B67">
         <v>23</v>
@@ -1939,12 +2140,15 @@
         <v>7</v>
       </c>
       <c r="F67">
+        <v>29</v>
+      </c>
+      <c r="G67">
         <v>47</v>
       </c>
     </row>
-    <row r="68" spans="1:6">
+    <row r="68" spans="1:7">
       <c r="A68" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B68">
         <v>23</v>
@@ -1959,12 +2163,15 @@
         <v>8</v>
       </c>
       <c r="F68">
+        <v>26</v>
+      </c>
+      <c r="G68">
         <v>48</v>
       </c>
     </row>
-    <row r="69" spans="1:6">
+    <row r="69" spans="1:7">
       <c r="A69" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B69">
         <v>23</v>
@@ -1979,12 +2186,15 @@
         <v>8</v>
       </c>
       <c r="F69">
+        <v>24</v>
+      </c>
+      <c r="G69">
         <v>48</v>
       </c>
     </row>
-    <row r="70" spans="1:6">
+    <row r="70" spans="1:7">
       <c r="A70" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B70">
         <v>23</v>
@@ -1999,12 +2209,15 @@
         <v>8</v>
       </c>
       <c r="F70">
+        <v>27</v>
+      </c>
+      <c r="G70">
         <v>48</v>
       </c>
     </row>
-    <row r="71" spans="1:6">
+    <row r="71" spans="1:7">
       <c r="A71" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B71">
         <v>23</v>
@@ -2019,6 +2232,9 @@
         <v>8</v>
       </c>
       <c r="F71">
+        <v>25</v>
+      </c>
+      <c r="G71">
         <v>48</v>
       </c>
     </row>

</xml_diff>